<commit_message>
Update ToolSelect UI labels, fix Mode B CoM MoI logic, unify CoG format, set defaults to 0
</commit_message>
<xml_diff>
--- a/InoRobotToolSelect/로봇 부하 및 로봇 선정 툴.xlsx
+++ b/InoRobotToolSelect/로봇 부하 및 로봇 선정 툴.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b96646d0fc390357/Desktop/made_C^N/InoRobotAssistant/InoRobotToolSelect/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="370" documentId="8_{FF835628-69DC-46F0-AE7A-65F4E0A80BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00198489-DA1B-4D32-A56D-F7BA10711283}"/>
+  <xr:revisionPtr revIDLastSave="371" documentId="8_{FF835628-69DC-46F0-AE7A-65F4E0A80BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{860E9803-1156-4FD7-9C2D-8A13C952B447}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="로봇 Tool 부하 선정" sheetId="1" r:id="rId1"/>
@@ -2251,6 +2251,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>